<commit_message>
R, sma, y graficos
</commit_message>
<xml_diff>
--- a/Bloque.xlsx
+++ b/Bloque.xlsx
@@ -845,10 +845,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
         <v>2</v>
@@ -872,7 +872,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G19" t="n">
         <v>4</v>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
@@ -1086,10 +1086,10 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>4</v>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E59" t="n">
         <v>1</v>
@@ -1792,7 +1792,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E61" t="n">
         <v>1</v>

</xml_diff>